<commit_message>
Update paths, model configurations, and change palette to Reds
</commit_message>
<xml_diff>
--- a/Data & Code/Kasus.xlsx
+++ b/Data & Code/Kasus.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30002"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lenovo\Downloads\Skripsi\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lenovo\Downloads\Skripsi\Data &amp; Code\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A0693282-0CD8-4392-891C-4F7077E3B502}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5A166CB-A5B5-4A99-B377-E9B1108F95DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2620" yWindow="2620" windowWidth="19200" windowHeight="9970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -132,7 +132,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -506,14 +506,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C28"/>
-  <sheetFormatPr defaultRowHeight="15.6"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.08203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.5" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="9.75" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -524,7 +524,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -535,7 +535,7 @@
         <v>5682300</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -546,7 +546,7 @@
         <v>2828020</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -557,7 +557,7 @@
         <v>2584990</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -568,7 +568,7 @@
         <v>3753120</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -579,7 +579,7 @@
         <v>2716950</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -590,7 +590,7 @@
         <v>1920920</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -601,7 +601,7 @@
         <v>1259230</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -612,7 +612,7 @@
         <v>1213930</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -623,7 +623,7 @@
         <v>2387960</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -634,7 +634,7 @@
         <v>1352540</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -645,7 +645,7 @@
         <v>1187130</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>14</v>
       </c>
@@ -656,7 +656,7 @@
         <v>1914040</v>
       </c>
     </row>
-    <row r="14" spans="1:3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>15</v>
       </c>
@@ -667,7 +667,7 @@
         <v>1663160</v>
       </c>
     </row>
-    <row r="15" spans="1:3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>16</v>
       </c>
@@ -678,7 +678,7 @@
         <v>1050340</v>
       </c>
     </row>
-    <row r="16" spans="1:3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>17</v>
       </c>
@@ -689,7 +689,7 @@
         <v>2554380</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>18</v>
       </c>
@@ -700,7 +700,7 @@
         <v>3273870</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>19</v>
       </c>
@@ -711,7 +711,7 @@
         <v>1884190</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>20</v>
       </c>
@@ -722,7 +722,7 @@
         <v>434100</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>21</v>
       </c>
@@ -733,7 +733,7 @@
         <v>1078350</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>22</v>
       </c>
@@ -744,7 +744,7 @@
         <v>365740</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>23</v>
       </c>
@@ -755,7 +755,7 @@
         <v>2528160</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>24</v>
       </c>
@@ -766,7 +766,7 @@
         <v>344850</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>25</v>
       </c>
@@ -777,7 +777,7 @@
         <v>2644060</v>
       </c>
     </row>
-    <row r="25" spans="1:3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>26</v>
       </c>
@@ -788,7 +788,7 @@
         <v>2163640</v>
       </c>
     </row>
-    <row r="26" spans="1:3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>27</v>
       </c>
@@ -799,7 +799,7 @@
         <v>598700</v>
       </c>
     </row>
-    <row r="27" spans="1:3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>28</v>
       </c>
@@ -810,7 +810,7 @@
         <v>750730</v>
       </c>
     </row>
-    <row r="28" spans="1:3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>29</v>
       </c>

</xml_diff>